<commit_message>
A lot to unpack here... The main change is I rewrote and with Claude.AI fixed the html report so it now saves one HTML per tab (with relative links between tabs). How plotly widgets are added to list has been cleaned up, which should make for more reliable displays and smaller lists. The lists are also not always kept in memory to save space, but reloaded when needed. The GSEA code was also rewritten to be parallelised and is thus much faster. The robustness of the code to occasional Shiny app issues has been increased. parClust is being checked more thoroughly now between runs against corruption, which should avoid having to recreate it so often. And lots of other micro changes...
</commit_message>
<xml_diff>
--- a/inst/extdata/LC_columns.xlsx
+++ b/inst/extdata/LC_columns.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\home\aRmel_package\proteoCraft\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3C4C644-76FC-4004-B877-0885D41EE7E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE18B3FE-EDE6-447D-A764-ACCF27652239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="131">
   <si>
     <t>Name</t>
   </si>
@@ -424,6 +424,9 @@
   </si>
   <si>
     <t>PepSep</t>
+  </si>
+  <si>
+    <t>Acquity Premier BEH C18</t>
   </si>
 </sst>
 </file>
@@ -1390,8 +1393,8 @@
       <c r="D17" s="4">
         <v>10</v>
       </c>
-      <c r="E17" s="4" t="s">
-        <v>60</v>
+      <c r="E17" s="4">
+        <v>2100</v>
       </c>
       <c r="F17" s="7">
         <v>2.7</v>
@@ -1417,7 +1420,7 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>87</v>
+        <v>130</v>
       </c>
       <c r="B18" t="s">
         <v>87</v>
@@ -1428,7 +1431,7 @@
       <c r="D18" s="4">
         <v>5</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="4">
         <v>2100</v>
       </c>
       <c r="F18" s="7" t="s">
@@ -1828,7 +1831,9 @@
       <c r="F29" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="G29" s="7"/>
+      <c r="G29" s="7" t="s">
+        <v>105</v>
+      </c>
       <c r="H29" t="s">
         <v>14</v>
       </c>
@@ -1864,7 +1869,9 @@
       <c r="F30" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="G30" s="7"/>
+      <c r="G30" s="7" t="s">
+        <v>105</v>
+      </c>
       <c r="H30" t="s">
         <v>14</v>
       </c>

</xml_diff>